<commit_message>
[MOSIP-43633] packetCreatedOn added in identity_schema (release-1.3x)
Signed-off-by: Nidhi0201 <nidhi.k@cyberpwn.com>
</commit_message>
<xml_diff>
--- a/mosip_master/xlsx/identity_schema.xlsx
+++ b/mosip_master/xlsx/identity_schema.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Project\Mosip\mosip-data\mosip_master\xlsx\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\mosip-data-fix-license\mosip_master\xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E632B33-EFBA-45CC-B1A2-807AF397E164}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D433272-7AFA-4B99-A709-E889310C4AF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="22620" windowHeight="13500" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -568,6 +568,14 @@
                     "fieldType": "default"
                 },
                 "typeOfDeath": {
+                    "bioAttributes": [
+                    ],
+                    "fieldCategory": "pvt",
+                    "format": "none",
+                    "type": "string",
+                    "fieldType": "default"
+                },
+				"packetCreatedOn": {
                     "bioAttributes": [
                     ],
                     "fieldCategory": "pvt",

</xml_diff>